<commit_message>
Corrected spelling in ABAI_P5_logbook.md and ensured Dockerfile uses Python 3.13-slim base image.
</commit_message>
<xml_diff>
--- a/P5_Maintenez_et_documentez_un_système_de_stockage_des_donnees_securise_et_performant_bailleul_aymeric/_projet/_docs/ABAI_P5_01_dico_donnees.xlsx
+++ b/P5_Maintenez_et_documentez_un_système_de_stockage_des_donnees_securise_et_performant_bailleul_aymeric/_projet/_docs/ABAI_P5_01_dico_donnees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mon Drive\_formation_over_git\P5_Maintenez_et_documentez_un_système_de_stockage_des_donnees_securise_et_performant_bailleul_aymeric\_projet\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB377ABD-B8AF-4B2D-A009-B29ACCA9609A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15501E0-BA2E-4F86-AE5E-29B8E25C6CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1335" yWindow="2940" windowWidth="36690" windowHeight="17940" xr2:uid="{99704DAC-E7D2-4A42-9EE7-A9262F7C8851}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{99704DAC-E7D2-4A42-9EE7-A9262F7C8851}"/>
   </bookViews>
   <sheets>
     <sheet name="patients" sheetId="1" r:id="rId1"/>
@@ -34,16 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
-  <si>
-    <t>Nom de la colonne</t>
-  </si>
-  <si>
-    <t>Type de donnée dans le CSV</t>
-  </si>
-  <si>
-    <t>Commentaire pour MongoDB</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="43">
   <si>
     <t>Name</t>
   </si>
@@ -51,109 +42,149 @@
     <t>String</t>
   </si>
   <si>
-    <t>Nom complet du patient.</t>
-  </si>
-  <si>
     <t>Age</t>
   </si>
   <si>
     <t>Integer</t>
   </si>
   <si>
-    <t>Âge du patient.</t>
-  </si>
-  <si>
     <t>Gender</t>
   </si>
   <si>
-    <t>Sexe du patient.</t>
-  </si>
-  <si>
     <t>Blood Type</t>
   </si>
   <si>
-    <t>Groupe sanguin.</t>
-  </si>
-  <si>
     <t>Medical Condition</t>
   </si>
   <si>
-    <t>Condition médicale principale.</t>
-  </si>
-  <si>
     <t>Date of Admission</t>
   </si>
   <si>
-    <t>String/Date</t>
-  </si>
-  <si>
-    <t>Convertir en type Date.</t>
-  </si>
-  <si>
     <t>Doctor</t>
   </si>
   <si>
-    <t>Nom du médecin traitant.</t>
-  </si>
-  <si>
     <t>Hospital</t>
   </si>
   <si>
-    <t>Nom de l'hôpital.</t>
-  </si>
-  <si>
     <t>Insurance Provider</t>
   </si>
   <si>
-    <t>Assureur.</t>
-  </si>
-  <si>
     <t>Billing Amount</t>
   </si>
   <si>
     <t>Float</t>
   </si>
   <si>
-    <t>Montant de la facturation.</t>
-  </si>
-  <si>
     <t>Room Number</t>
   </si>
   <si>
-    <t>Numéro de chambre.</t>
-  </si>
-  <si>
     <t>Admission Type</t>
   </si>
   <si>
-    <t>Type d'admission (Urgent, Elective, Emergency).</t>
-  </si>
-  <si>
     <t>Discharge Date</t>
   </si>
   <si>
     <t>Medication</t>
   </si>
   <si>
-    <t>Médicament prescrit.</t>
-  </si>
-  <si>
     <t>Test Results</t>
   </si>
   <si>
-    <t>Résultat des tests.</t>
-  </si>
-  <si>
-    <t>Table Patients</t>
+    <t>CODE</t>
+  </si>
+  <si>
+    <t>TYPE</t>
+  </si>
+  <si>
+    <t>NATURE</t>
+  </si>
+  <si>
+    <t>REGLE DE GESTION</t>
+  </si>
+  <si>
+    <t>REGLE DE CALCUL</t>
+  </si>
+  <si>
+    <t>SIGNIFICATION</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Date d'admission</t>
+  </si>
+  <si>
+    <t>Date de sortie</t>
+  </si>
+  <si>
+    <t>Elémentaire</t>
+  </si>
+  <si>
+    <t>Convertir en type Date</t>
+  </si>
+  <si>
+    <t>Nom complet du patient</t>
+  </si>
+  <si>
+    <t>Âge du patient</t>
+  </si>
+  <si>
+    <t>Sexe du patient</t>
+  </si>
+  <si>
+    <t>Groupe sanguin</t>
+  </si>
+  <si>
+    <t>Condition médicale principale</t>
+  </si>
+  <si>
+    <t>Nom du médecin traitant</t>
+  </si>
+  <si>
+    <t>Nom de l'hôpital</t>
+  </si>
+  <si>
+    <t>Assureur</t>
+  </si>
+  <si>
+    <t>Montant de la facturation</t>
+  </si>
+  <si>
+    <t>Numéro de chambre</t>
+  </si>
+  <si>
+    <t>Type d'admission (Urgent, Elective, Emergency)</t>
+  </si>
+  <si>
+    <t>Médicament prescrit</t>
+  </si>
+  <si>
+    <t>Résultat des tests</t>
+  </si>
+  <si>
+    <t>Dico patients</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -182,7 +213,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -203,12 +234,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FA3E4E7E-B657-4A95-8A50-EC6208DE2243}" name="Tableau2" displayName="Tableau2" ref="A2:C17" totalsRowShown="0">
-  <autoFilter ref="A2:C17" xr:uid="{FA3E4E7E-B657-4A95-8A50-EC6208DE2243}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{2F0E3711-1D47-4AA4-B6CB-228232B55713}" name="Nom de la colonne"/>
-    <tableColumn id="2" xr3:uid="{113FBD40-509F-4D2D-AC8C-4279F907FAD7}" name="Type de donnée dans le CSV"/>
-    <tableColumn id="3" xr3:uid="{A8048265-02B0-4019-831B-59D01266C360}" name="Commentaire pour MongoDB"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FA3E4E7E-B657-4A95-8A50-EC6208DE2243}" name="Tableau2" displayName="Tableau2" ref="A2:F17" totalsRowShown="0">
+  <autoFilter ref="A2:F17" xr:uid="{FA3E4E7E-B657-4A95-8A50-EC6208DE2243}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{2F0E3711-1D47-4AA4-B6CB-228232B55713}" name="CODE"/>
+    <tableColumn id="4" xr3:uid="{AEA0CA2F-5B3C-44BC-8DFA-D88EC257CE5C}" name="SIGNIFICATION"/>
+    <tableColumn id="8" xr3:uid="{14913933-05E4-49C8-8B3D-F605A6521290}" name="TYPE"/>
+    <tableColumn id="6" xr3:uid="{3CCCB3B9-3547-4C5E-93D3-12D6015B0E14}" name="NATURE"/>
+    <tableColumn id="3" xr3:uid="{A8048265-02B0-4019-831B-59D01266C360}" name="REGLE DE GESTION"/>
+    <tableColumn id="7" xr3:uid="{D902C24E-2EEF-49E0-ABE8-0DEED2A0F9CA}" name="REGLE DE CALCUL"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -511,204 +545,279 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{288B7831-7B80-4335-B003-1E1F280A9909}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="22.7109375" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="22.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-    </row>
-    <row r="2" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>16</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>34</v>
-      </c>
       <c r="B17" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3:C17" xr:uid="{B9E76A7F-B588-4F40-B530-C5BDFA98309B}">
+      <formula1>"String,Integer,Date,Float"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D3:D17" xr:uid="{C6197F86-C021-437B-AC9D-457B2EC668E3}">
+      <formula1>"???,Elémentaire,Calculé,Concatété,Primary key,Foreign key,"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>